<commit_message>
Update der To Do Liste
</commit_message>
<xml_diff>
--- a/CASESTUDY_Hydrogenation.xlsx
+++ b/CASESTUDY_Hydrogenation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://universityofcambridgecloud-my.sharepoint.com/personal/lf576_cam_ac_uk/Documents/04_Coding/hydrogenation/current_versions/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="35" documentId="8_{3CA0C22B-1C3C-468B-A8A4-EC46740A7B5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{376BE0CC-9E22-4B97-BA0E-DE8BF9F43929}"/>
+  <xr:revisionPtr revIDLastSave="54" documentId="8_{3CA0C22B-1C3C-468B-A8A4-EC46740A7B5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E697BDC1-13ED-4EBC-B1A3-01FB133D5D2F}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="3" xr2:uid="{D5389695-9B6E-4686-BC98-C44AC3042CAD}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
     <sheet name="Overview" sheetId="2" r:id="rId2"/>
     <sheet name="CaseStudy_Hydrogenation" sheetId="3" r:id="rId3"/>
-    <sheet name="Context_Hydrogenation_New" sheetId="4" r:id="rId4"/>
+    <sheet name="Context_Input" sheetId="4" r:id="rId4"/>
     <sheet name="Context_Compact" sheetId="5" r:id="rId5"/>
     <sheet name="Context Hydrogenation" sheetId="6" r:id="rId6"/>
   </sheets>
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="845" uniqueCount="486">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="849" uniqueCount="492">
   <si>
     <t>This is the file containing all the information about the Hydrogenation Process Case Study</t>
   </si>
@@ -911,9 +911,6 @@
     <t>#CoolingFluidStream</t>
   </si>
   <si>
-    <t>Setze ich das flowrate profile hierhin oder an die jacket oder an den Stream (Stream dann ohne Kontext)</t>
-  </si>
-  <si>
     <t>#Jacket_Structure</t>
   </si>
   <si>
@@ -968,9 +965,6 @@
     <t>Wenn ich den Space der Phase mit dem MaterialVolume beschreibe, brauche ich dann überhaupt die Vessel noch? Weil dann wissen wir ja MaterialVolume Reactor locatedIn Vessel</t>
   </si>
   <si>
-    <t>Die Initial Mass Fractions hier oder in die Molekül Contexts</t>
-  </si>
-  <si>
     <t>#LiquidPhase</t>
   </si>
   <si>
@@ -1524,13 +1518,37 @@
   </si>
   <si>
     <t>#H4</t>
+  </si>
+  <si>
+    <t>In Context_Input können die Devices, Phases und Molecules eingefügt werden, und dann kann man direkt deren Kontext beschreiben</t>
+  </si>
+  <si>
+    <t>Daraufhin wird automatisch der kompakte Kontext in Context_Compact erstellt</t>
+  </si>
+  <si>
+    <t>Diesen kann man dann rauskopieren in die Excel context_connections.xlsx</t>
+  </si>
+  <si>
+    <t>Wenn man dann  python create_context_connections.py aufruft, erstellt es einem automatisch die entsprechenden Connections mit den Properties, die dann in das RO-Crate eingefügt werden können</t>
+  </si>
+  <si>
+    <t>Für das Einfügen habe ich bis jetzt noch keine Automatisierungsschritt erstellt.</t>
+  </si>
+  <si>
+    <t>#InitialMassFraction_Water_LiquidPhase in Liquid Phase</t>
+  </si>
+  <si>
+    <t>#SetFlowrateProfile_Jacket in Jacket</t>
+  </si>
+  <si>
+    <t>Reactor Energy würde ich prinzipiell nicht wirklich hiermit verbinden, aber da ich definiert habe dass MassFlowMeter ein Teil von Reactor ist muss ich das der Vollständigkeit halber auch hier aufführen</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1554,6 +1572,12 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1627,7 +1651,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -1649,6 +1673,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1983,12 +2008,37 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30D6EF24-A5F2-4E49-9641-E94D8B75807A}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:A7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>488</v>
       </c>
     </row>
   </sheetData>
@@ -3713,7 +3763,7 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="B1" t="s">
         <v>243</v>
@@ -3734,13 +3784,13 @@
         <v>233</v>
       </c>
       <c r="H1" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="I1" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="J1" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
     </row>
     <row r="2" spans="1:10" s="11" customFormat="1" x14ac:dyDescent="0.25"/>
@@ -3754,74 +3804,74 @@
     </row>
     <row r="4" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="B4" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="C4" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="D4" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="H4" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
     </row>
     <row r="5" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="B5" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="C5" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="D5" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="H5" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
     </row>
     <row r="6" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>360</v>
+      </c>
+      <c r="B6" t="s">
+        <v>363</v>
+      </c>
+      <c r="C6" t="s">
         <v>362</v>
       </c>
-      <c r="B6" t="s">
-        <v>365</v>
-      </c>
-      <c r="C6" t="s">
-        <v>364</v>
-      </c>
       <c r="D6" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="H6" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
     </row>
     <row r="7" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="C7" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="H7" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="8" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H8" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
     </row>
     <row r="9" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H9" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
     </row>
     <row r="10" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25"/>
@@ -3831,7 +3881,7 @@
     <row r="14" spans="1:10" s="11" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="15" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="J15" s="2" t="s">
         <v>90</v>
@@ -3839,48 +3889,48 @@
     </row>
     <row r="16" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="B16" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="C16" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="D16" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="H16" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
     </row>
     <row r="17" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="B17" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="H17" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
     </row>
     <row r="18" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H18" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
     </row>
     <row r="19" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H19" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="20" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H20" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
     </row>
     <row r="21" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25"/>
@@ -3903,61 +3953,61 @@
     </row>
     <row r="29" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="B29" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="C29" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="D29" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="H29" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
     </row>
     <row r="30" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="B30" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="C30" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="D30" s="7" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="H30" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
     </row>
     <row r="31" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H31" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
     </row>
     <row r="32" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H32" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="33" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H33" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
     </row>
     <row r="34" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H34" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
     </row>
     <row r="35" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H35" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
     </row>
     <row r="36" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25"/>
@@ -3975,51 +4025,51 @@
     </row>
     <row r="42" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="B42" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="C42" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="D42" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="H42" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
     </row>
     <row r="43" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="B43" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="C43" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="D43" s="7" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="H43" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
     </row>
     <row r="44" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H44" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
     </row>
     <row r="45" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H45" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="46" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H46" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
     </row>
     <row r="47" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25"/>
@@ -4039,51 +4089,51 @@
     </row>
     <row r="55" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="B55" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="C55" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="D55" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="H55" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
     </row>
     <row r="56" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="B56" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="C56" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="D56" s="7" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="H56" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
     </row>
     <row r="57" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H57" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
     </row>
     <row r="58" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H58" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="59" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H59" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
     </row>
     <row r="60" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25"/>
@@ -4095,7 +4145,7 @@
     <row r="66" spans="1:10" s="11" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="67" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="J67" s="2" t="s">
         <v>90</v>
@@ -4103,51 +4153,51 @@
     </row>
     <row r="68" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="B68" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="C68" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="D68" s="7" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="H68" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
     </row>
     <row r="69" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="B69" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="C69" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="D69" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="H69" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
     </row>
     <row r="70" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H70" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
     </row>
     <row r="71" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H71" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="72" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H72" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
     </row>
     <row r="73" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25"/>
@@ -4159,7 +4209,7 @@
     <row r="79" spans="1:10" s="11" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="80" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="J80" s="2" t="s">
         <v>90</v>
@@ -4167,51 +4217,51 @@
     </row>
     <row r="81" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="B81" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="C81" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="D81" s="7" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="H81" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="82" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="B82" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="C82" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="D82" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="H82" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
     </row>
     <row r="83" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H83" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
     </row>
     <row r="84" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H84" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="85" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H85" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
     </row>
     <row r="86" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25"/>
@@ -4223,7 +4273,7 @@
     <row r="92" spans="1:10" s="11" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="93" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A93" s="2" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="J93" s="2" t="s">
         <v>90</v>
@@ -4231,51 +4281,54 @@
     </row>
     <row r="94" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="B94" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="C94" s="7" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="D94" s="7" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="H94" t="s">
-        <v>315</v>
+        <v>313</v>
+      </c>
+      <c r="I94" t="s">
+        <v>491</v>
       </c>
     </row>
     <row r="95" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="B95" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="C95" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="D95" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="H95" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
     </row>
     <row r="96" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H96" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
     </row>
     <row r="97" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H97" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="98" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H98" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
     </row>
     <row r="99" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25"/>
@@ -4287,7 +4340,7 @@
     <row r="105" spans="1:10" s="11" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="106" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A106" s="2" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="J106" s="2" t="s">
         <v>90</v>
@@ -4295,42 +4348,42 @@
     </row>
     <row r="107" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="B107" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="D107" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="H107" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
     </row>
     <row r="108" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="B108" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="H108" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
     </row>
     <row r="109" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H109" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
     </row>
     <row r="110" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H110" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="111" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H111" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
     </row>
     <row r="112" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25"/>
@@ -4354,27 +4407,27 @@
     </row>
     <row r="124" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="C124" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="E124" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="G124" t="s">
         <v>261</v>
       </c>
       <c r="I124" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
     </row>
     <row r="125" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="E125" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="G125" t="s">
         <v>266</v>
@@ -4382,21 +4435,18 @@
     </row>
     <row r="126" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="E126" t="s">
-        <v>288</v>
-      </c>
-      <c r="I126" t="s">
-        <v>299</v>
+        <v>287</v>
       </c>
     </row>
     <row r="127" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="E127" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="128" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25"/>
@@ -4417,32 +4467,32 @@
     </row>
     <row r="137" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C137" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="E137" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="G137" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="138" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="E138" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="139" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="E139" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="140" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25"/>
@@ -4464,29 +4514,29 @@
     </row>
     <row r="150" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C150" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="E150" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="151" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="E151" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="152" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="E152" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="153" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25"/>
@@ -4508,29 +4558,29 @@
     </row>
     <row r="163" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C163" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="E163" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="164" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="E164" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="165" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="E165" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="166" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25"/>
@@ -4544,7 +4594,7 @@
     <row r="174" spans="1:10" s="11" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="175" spans="1:10" s="13" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A175" s="13" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="J175" s="13" t="s">
         <v>89</v>
@@ -4552,29 +4602,29 @@
     </row>
     <row r="176" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C176" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="E176" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="177" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="E177" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="178" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="E178" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="179" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25"/>
@@ -4588,7 +4638,7 @@
     <row r="187" spans="1:10" s="11" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="188" spans="1:10" s="13" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A188" s="13" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="J188" s="13" t="s">
         <v>89</v>
@@ -4596,32 +4646,29 @@
     </row>
     <row r="189" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="C189" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="E189" t="s">
-        <v>284</v>
+        <v>283</v>
+      </c>
+      <c r="I189" s="15" t="s">
+        <v>490</v>
       </c>
     </row>
     <row r="190" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
-        <v>286</v>
-      </c>
-      <c r="C190" s="7" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="E190" t="s">
-        <v>282</v>
-      </c>
-      <c r="I190" t="s">
         <v>281</v>
       </c>
     </row>
     <row r="191" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="E191" t="s">
         <v>280</v>
@@ -4725,7 +4772,7 @@
     </row>
     <row r="232" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
       <c r="C232" t="s">
         <v>269</v>
@@ -4733,7 +4780,7 @@
     </row>
     <row r="233" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="C233" t="s">
         <v>268</v>
@@ -4766,12 +4813,11 @@
       <c r="E244" t="s">
         <v>262</v>
       </c>
-    </row>
-    <row r="245" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="E245" s="7" t="s">
-        <v>266</v>
-      </c>
-    </row>
+      <c r="I244" s="15" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="245" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25"/>
     <row r="246" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25"/>
     <row r="247" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25"/>
     <row r="248" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25"/>
@@ -4800,12 +4846,11 @@
       <c r="E257" t="s">
         <v>262</v>
       </c>
-    </row>
-    <row r="258" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="E258" s="7" t="s">
+      <c r="I257" s="15" t="s">
         <v>261</v>
       </c>
     </row>
+    <row r="258" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25"/>
     <row r="259" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25"/>
     <row r="260" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25"/>
     <row r="261" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25"/>
@@ -5021,9 +5066,9 @@
     <row r="366" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25"/>
     <row r="367" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25"/>
     <row r="368" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25"/>
-    <row r="369" customFormat="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
-    <row r="370" customFormat="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
-    <row r="371" customFormat="1" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="369" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="370" outlineLevel="1" x14ac:dyDescent="0.25"/>
+    <row r="371" outlineLevel="1" x14ac:dyDescent="0.25"/>
     <row r="372" s="9" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="373" s="9" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="374" s="9" customFormat="1" x14ac:dyDescent="0.25"/>
@@ -5040,7 +5085,7 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="B1" t="s">
         <v>243</v>
@@ -5063,7 +5108,7 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="str" cm="1">
-        <f t="array" ref="A2:G11">Context_Hydrogenation_New!A4:G13</f>
+        <f t="array" ref="A2:G11">Context_Input!A4:G13</f>
         <v>#Reactor</v>
       </c>
       <c r="B2" t="str">
@@ -5294,7 +5339,7 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="str" cm="1">
-        <f t="array" ref="A12:G22">Context_Hydrogenation_New!A16:G26</f>
+        <f t="array" ref="A12:G22">Context_Input!A16:G26</f>
         <v>#Vessel</v>
       </c>
       <c r="B12" t="str">
@@ -5548,7 +5593,7 @@
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="str" cm="1">
-        <f t="array" ref="A23:G33">Context_Hydrogenation_New!A29:G39</f>
+        <f t="array" ref="A23:G33">Context_Input!A29:G39</f>
         <v>#Stirrer</v>
       </c>
       <c r="B23" t="str">
@@ -5802,7 +5847,7 @@
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" t="str" cm="1">
-        <f t="array" ref="A34:G44">Context_Hydrogenation_New!A42:G52</f>
+        <f t="array" ref="A34:G44">Context_Input!A42:G52</f>
         <v>#Sparger</v>
       </c>
       <c r="B34" t="str">
@@ -6056,7 +6101,7 @@
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" t="str" cm="1">
-        <f t="array" ref="A45:G55">Context_Hydrogenation_New!A55:G65</f>
+        <f t="array" ref="A45:G55">Context_Input!A55:G65</f>
         <v>#Jacket</v>
       </c>
       <c r="B45" t="str">
@@ -6310,7 +6355,7 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" t="str" cm="1">
-        <f t="array" ref="A56:G66">Context_Hydrogenation_New!A68:G78</f>
+        <f t="array" ref="A56:G66">Context_Input!A68:G78</f>
         <v>#TemperatureSensor</v>
       </c>
       <c r="B56" t="str">
@@ -6564,7 +6609,7 @@
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67" t="str" cm="1">
-        <f t="array" ref="A67:G77">Context_Hydrogenation_New!A81:G91</f>
+        <f t="array" ref="A67:G77">Context_Input!A81:G91</f>
         <v>#PressureSensor</v>
       </c>
       <c r="B67" t="str">
@@ -6818,7 +6863,7 @@
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A78" t="str" cm="1">
-        <f t="array" ref="A78:G88">Context_Hydrogenation_New!A94:G104</f>
+        <f t="array" ref="A78:G88">Context_Input!A94:G104</f>
         <v>#MassFlowMeter</v>
       </c>
       <c r="B78" t="str">
@@ -7072,7 +7117,7 @@
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A89" t="str" cm="1">
-        <f t="array" ref="A89:G100">Context_Hydrogenation_New!A107:G118</f>
+        <f t="array" ref="A89:G100">Context_Input!A107:G118</f>
         <v>#Balance</v>
       </c>
       <c r="B89" t="str">
@@ -7349,7 +7394,7 @@
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A101" t="str" cm="1">
-        <f t="array" ref="A101:G111">Context_Hydrogenation_New!A124:G134</f>
+        <f t="array" ref="A101:G111">Context_Input!A124:G134</f>
         <v>#LiquidPhase</v>
       </c>
       <c r="B101">
@@ -7603,7 +7648,7 @@
     </row>
     <row r="112" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A112" t="str" cm="1">
-        <f t="array" ref="A112:G122">Context_Hydrogenation_New!A137:G147</f>
+        <f t="array" ref="A112:G122">Context_Input!A137:G147</f>
         <v>#SolidPhase</v>
       </c>
       <c r="B112">
@@ -7857,7 +7902,7 @@
     </row>
     <row r="123" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A123" t="str" cm="1">
-        <f t="array" ref="A123:G133">Context_Hydrogenation_New!A150:G160</f>
+        <f t="array" ref="A123:G133">Context_Input!A150:G160</f>
         <v>#CatalystPhase</v>
       </c>
       <c r="B123">
@@ -8111,7 +8156,7 @@
     </row>
     <row r="134" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A134" t="str" cm="1">
-        <f t="array" ref="A134:G144">Context_Hydrogenation_New!A163:G173</f>
+        <f t="array" ref="A134:G144">Context_Input!A163:G173</f>
         <v>#GasPhase</v>
       </c>
       <c r="B134">
@@ -8365,7 +8410,7 @@
     </row>
     <row r="145" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A145" t="str" cm="1">
-        <f t="array" ref="A145:G155">Context_Hydrogenation_New!A176:G186</f>
+        <f t="array" ref="A145:G155">Context_Input!A176:G186</f>
         <v>#DispersedGasPhase</v>
       </c>
       <c r="B145">
@@ -8619,7 +8664,7 @@
     </row>
     <row r="156" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A156" t="str" cm="1">
-        <f t="array" ref="A156:G166">Context_Hydrogenation_New!A189:G199</f>
+        <f t="array" ref="A156:G166">Context_Input!A189:G199</f>
         <v>#CoolingFluidPhase</v>
       </c>
       <c r="B156">
@@ -8648,8 +8693,8 @@
       <c r="B157">
         <v>0</v>
       </c>
-      <c r="C157" t="str">
-        <v>#SetFlowrateProfile_Jacket</v>
+      <c r="C157">
+        <v>0</v>
       </c>
       <c r="D157">
         <v>0</v>
@@ -8873,7 +8918,7 @@
     </row>
     <row r="167" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A167" t="str" cm="1">
-        <f t="array" ref="A167:G177">Context_Hydrogenation_New!A202:G212</f>
+        <f t="array" ref="A167:G177">Context_Input!A202:G212</f>
         <v>#HydrogenSpargerPhase</v>
       </c>
       <c r="B167">
@@ -9127,7 +9172,7 @@
     </row>
     <row r="178" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A178" t="str" cm="1">
-        <f t="array" ref="A178:G188">Context_Hydrogenation_New!A215:G225</f>
+        <f t="array" ref="A178:G188">Context_Input!A215:G225</f>
         <v>#CleaningFluidPhase</v>
       </c>
       <c r="B178">
@@ -9381,7 +9426,7 @@
     </row>
     <row r="189" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A189" t="str" cm="1">
-        <f t="array" ref="A189:G199">Context_Hydrogenation_New!A231:G241</f>
+        <f t="array" ref="A189:G199">Context_Input!A231:G241</f>
         <v>#H2</v>
       </c>
       <c r="B189">
@@ -9635,7 +9680,7 @@
     </row>
     <row r="200" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A200" t="str" cm="1">
-        <f t="array" ref="A200:G210">Context_Hydrogenation_New!A244:G254</f>
+        <f t="array" ref="A200:G210">Context_Input!A244:G254</f>
         <v>#H2O</v>
       </c>
       <c r="B200">
@@ -9670,8 +9715,8 @@
       <c r="D201">
         <v>0</v>
       </c>
-      <c r="E201" t="str">
-        <v>#InitialMassFraction_Water_LiquidPhase</v>
+      <c r="E201">
+        <v>0</v>
       </c>
       <c r="F201">
         <v>0</v>
@@ -9889,7 +9934,7 @@
     </row>
     <row r="211" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A211" t="str" cm="1">
-        <f t="array" ref="A211:G221">Context_Hydrogenation_New!A257:G267</f>
+        <f t="array" ref="A211:G221">Context_Input!A257:G267</f>
         <v>#Solvent</v>
       </c>
       <c r="B211">
@@ -9924,8 +9969,8 @@
       <c r="D212">
         <v>0</v>
       </c>
-      <c r="E212" t="str">
-        <v>#InitialMassFraction_Solvent_LiquidPhase</v>
+      <c r="E212">
+        <v>0</v>
       </c>
       <c r="F212">
         <v>0</v>
@@ -10143,7 +10188,7 @@
     </row>
     <row r="222" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A222" t="str" cm="1">
-        <f t="array" ref="A222:G232">Context_Hydrogenation_New!A270:G280</f>
+        <f t="array" ref="A222:G232">Context_Input!A270:G280</f>
         <v>#RDY</v>
       </c>
       <c r="B222">
@@ -10397,7 +10442,7 @@
     </row>
     <row r="233" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A233" cm="1">
-        <f t="array" ref="A233:G243">Context_Hydrogenation_New!A283:G293</f>
+        <f t="array" ref="A233:G243">Context_Input!A283:G293</f>
         <v>0</v>
       </c>
       <c r="B233">
@@ -10651,7 +10696,7 @@
     </row>
     <row r="244" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A244" cm="1">
-        <f t="array" ref="A244:G254">Context_Hydrogenation_New!A296:G306</f>
+        <f t="array" ref="A244:G254">Context_Input!A296:G306</f>
         <v>0</v>
       </c>
       <c r="B244">
@@ -10905,7 +10950,7 @@
     </row>
     <row r="255" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A255" cm="1">
-        <f t="array" ref="A255:G265">Context_Hydrogenation_New!A309:G319</f>
+        <f t="array" ref="A255:G265">Context_Input!A309:G319</f>
         <v>0</v>
       </c>
       <c r="B255">
@@ -11159,7 +11204,7 @@
     </row>
     <row r="266" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A266" t="str" cm="1">
-        <f t="array" ref="A266:G276">Context_Hydrogenation_New!A322:G332</f>
+        <f t="array" ref="A266:G276">Context_Input!A322:G332</f>
         <v>#RDEt</v>
       </c>
       <c r="B266">
@@ -11413,7 +11458,7 @@
     </row>
     <row r="277" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A277" t="str" cm="1">
-        <f t="array" ref="A277:G287">Context_Hydrogenation_New!A335:G345</f>
+        <f t="array" ref="A277:G287">Context_Input!A335:G345</f>
         <v>#Dimer1</v>
       </c>
       <c r="B277">
@@ -11667,7 +11712,7 @@
     </row>
     <row r="288" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A288" t="str" cm="1">
-        <f t="array" ref="A288:G298">Context_Hydrogenation_New!A348:G358</f>
+        <f t="array" ref="A288:G298">Context_Input!A348:G358</f>
         <v>#Dimer2</v>
       </c>
       <c r="B288">
@@ -11921,7 +11966,7 @@
     </row>
     <row r="299" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A299" t="str" cm="1">
-        <f t="array" ref="A299:G309">Context_Hydrogenation_New!A361:G371</f>
+        <f t="array" ref="A299:G309">Context_Input!A361:G371</f>
         <v>#Pt</v>
       </c>
       <c r="B299">
@@ -12193,47 +12238,47 @@
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="B1" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="C1" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
       <c r="D1" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="E1" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="B2" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="K2" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="B4" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="C4" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="L4" s="14" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="M4" s="14"/>
       <c r="N4" s="14"/>
@@ -12241,16 +12286,16 @@
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="K5" s="5"/>
       <c r="L5" s="5" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="M5" s="5" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="N5" s="5" t="s">
         <v>90</v>
       </c>
       <c r="O5" s="5" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="Q5" t="s">
         <v>243</v>
@@ -12258,22 +12303,22 @@
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="B6" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="E6" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
       <c r="K6" s="11" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
       <c r="L6" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
       <c r="M6" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="Q6" t="s">
         <v>241</v>
@@ -12281,22 +12326,22 @@
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>459</v>
+      </c>
+      <c r="B7" t="s">
+        <v>464</v>
+      </c>
+      <c r="E7" t="s">
+        <v>463</v>
+      </c>
+      <c r="K7" s="11" t="s">
+        <v>462</v>
+      </c>
+      <c r="L7" t="s">
         <v>461</v>
       </c>
-      <c r="B7" t="s">
-        <v>466</v>
-      </c>
-      <c r="E7" t="s">
-        <v>465</v>
-      </c>
-      <c r="K7" s="11" t="s">
-        <v>464</v>
-      </c>
-      <c r="L7" t="s">
-        <v>463</v>
-      </c>
       <c r="M7" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="Q7" t="s">
         <v>239</v>
@@ -12304,25 +12349,25 @@
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="B8" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="E8" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
       <c r="K8" s="11" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="L8" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="M8" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="N8" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="Q8" t="s">
         <v>237</v>
@@ -12333,13 +12378,13 @@
         <v>250</v>
       </c>
       <c r="B9" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
       <c r="K9" s="11" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
       <c r="M9" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
       <c r="Q9" t="s">
         <v>235</v>
@@ -12347,16 +12392,16 @@
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="B10" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
       <c r="K10" s="11" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="M10" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="Q10" t="s">
         <v>233</v>
@@ -12367,10 +12412,10 @@
         <v>258</v>
       </c>
       <c r="B11" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="K11" s="11" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="M11" t="s">
         <v>241</v>
@@ -12381,7 +12426,7 @@
         <v>261</v>
       </c>
       <c r="B12" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="K12" s="11" t="s">
         <v>89</v>
@@ -12392,7 +12437,7 @@
         <v>266</v>
       </c>
       <c r="B13" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="K13" s="11" t="s">
         <v>248</v>
@@ -12400,141 +12445,141 @@
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B14" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="K14" s="11" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="L14" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="M14" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="N14" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="O14" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="B15" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="E15" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="K15" s="11" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="N15" t="s">
         <v>243</v>
       </c>
       <c r="O15" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="B16" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="K16" s="11" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B17" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="D17" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="K17" s="11" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="M17" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="B18" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="E18" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="K18" s="11" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="M18" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="N18" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="B19" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="K19" s="11" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="N19" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="O19" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="B20" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="K20" s="11" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="M20" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="N20" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="B21" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="D21" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="K21" s="11" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="M21" t="s">
         <v>233</v>
@@ -12542,19 +12587,19 @@
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="B22" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="K22" s="11" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="L22" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="M22" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="N22" t="s">
         <v>239</v>
@@ -12562,223 +12607,223 @@
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="E23" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="B24" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="E24" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="B25" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="E25" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="B26" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="E26" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="B27" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="E27" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="B28" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="E28" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="B29" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="B30" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="B31" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.25">
       <c r="E32" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="B33" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="E33" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="B34" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="E34" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="B35" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="B36" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="B37" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="E37" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="B38" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="B39" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="B40" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B41" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="B42" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="B43" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="B44" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="B45" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="B46" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="B47" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
anpassen der create_context_connection python file, da die im Output nur die IDs hintereinander geschrieben hat ohne echte Verlinkung
</commit_message>
<xml_diff>
--- a/CASESTUDY_Hydrogenation.xlsx
+++ b/CASESTUDY_Hydrogenation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://universityofcambridgecloud-my.sharepoint.com/personal/lf576_cam_ac_uk/Documents/04_Coding/hydrogenation/current_versions/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="59" documentId="8_{3CA0C22B-1C3C-468B-A8A4-EC46740A7B5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5F8180BA-4D06-4597-B6A5-06D2096C39F6}"/>
+  <xr:revisionPtr revIDLastSave="61" documentId="8_{3CA0C22B-1C3C-468B-A8A4-EC46740A7B5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9B5A8AA5-601C-4729-92E8-464BFE446E83}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{D5389695-9B6E-4686-BC98-C44AC3042CAD}"/>
   </bookViews>
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="849" uniqueCount="492">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="849" uniqueCount="490">
   <si>
     <t>This is the file containing all the information about the Hydrogenation Process Case Study</t>
   </si>
@@ -1512,12 +1512,6 @@
   </si>
   <si>
     <t>describes Context</t>
-  </si>
-  <si>
-    <t>#H3</t>
-  </si>
-  <si>
-    <t>#H4</t>
   </si>
   <si>
     <t>In Context_Input können die Devices, Phases und Molecules eingefügt werden, und dann kann man direkt deren Kontext beschreiben</t>
@@ -2034,27 +2028,27 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
     </row>
   </sheetData>
@@ -4335,7 +4329,7 @@
         <v>313</v>
       </c>
       <c r="I94" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
     </row>
     <row r="95" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.3">
@@ -4721,7 +4715,7 @@
         <v>283</v>
       </c>
       <c r="I189" s="14" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
     </row>
     <row r="190" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.3">
@@ -4853,7 +4847,7 @@
     </row>
     <row r="232" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A232" t="s">
-        <v>482</v>
+        <v>115</v>
       </c>
       <c r="C232" t="s">
         <v>269</v>
@@ -4861,7 +4855,7 @@
     </row>
     <row r="233" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A233" t="s">
-        <v>483</v>
+        <v>115</v>
       </c>
       <c r="C233" t="s">
         <v>268</v>
@@ -4898,7 +4892,7 @@
         <v>262</v>
       </c>
       <c r="I244" s="14" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
     </row>
     <row r="245" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.3"/>
@@ -9567,7 +9561,7 @@
     </row>
     <row r="190" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A190" t="str">
-        <v>#H3</v>
+        <v>#H2</v>
       </c>
       <c r="B190">
         <v>0</v>
@@ -9590,7 +9584,7 @@
     </row>
     <row r="191" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A191" t="str">
-        <v>#H4</v>
+        <v>#H2</v>
       </c>
       <c r="B191">
         <v>0</v>

</xml_diff>

<commit_message>
Hinzufügen des neuen Kontexts und bereinigen der Datei
</commit_message>
<xml_diff>
--- a/CASESTUDY_Hydrogenation.xlsx
+++ b/CASESTUDY_Hydrogenation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://universityofcambridgecloud-my.sharepoint.com/personal/lf576_cam_ac_uk/Documents/04_Coding/hydrogenation/current_versions/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="77" documentId="8_{3CA0C22B-1C3C-468B-A8A4-EC46740A7B5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C125219F-38CE-4786-915C-CFB519907254}"/>
+  <xr:revisionPtr revIDLastSave="82" documentId="8_{3CA0C22B-1C3C-468B-A8A4-EC46740A7B5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BF7C0A2E-C8D9-446A-BC72-41ADC02F7BB1}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="3" xr2:uid="{D5389695-9B6E-4686-BC98-C44AC3042CAD}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="861" uniqueCount="493">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="864" uniqueCount="492">
   <si>
     <t>This is the file containing all the information about the Hydrogenation Process Case Study</t>
   </si>
@@ -831,9 +831,6 @@
   </si>
   <si>
     <t>Dimer1</t>
-  </si>
-  <si>
-    <t>#FinalMassRDEt</t>
   </si>
   <si>
     <t>#RDEt</t>
@@ -2041,27 +2038,27 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
     </row>
   </sheetData>
@@ -3786,7 +3783,7 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="B1" t="s">
         <v>243</v>
@@ -3807,13 +3804,13 @@
         <v>233</v>
       </c>
       <c r="H1" s="16" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="I1" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="J1" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
     </row>
     <row r="2" spans="1:10" s="11" customFormat="1" x14ac:dyDescent="0.25">
@@ -3830,74 +3827,74 @@
     </row>
     <row r="4" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="B4" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="C4" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="D4" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="H4" s="16" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="B5" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="C5" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="D5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="H5" s="16" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>359</v>
+      </c>
+      <c r="B6" t="s">
+        <v>362</v>
+      </c>
+      <c r="C6" t="s">
+        <v>361</v>
+      </c>
+      <c r="D6" t="s">
         <v>360</v>
       </c>
-      <c r="B6" t="s">
-        <v>363</v>
-      </c>
-      <c r="C6" t="s">
-        <v>362</v>
-      </c>
-      <c r="D6" t="s">
-        <v>361</v>
-      </c>
       <c r="H6" s="16" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="C7" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="H7" s="16" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H8" s="16" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H9" s="16" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25"/>
@@ -3909,7 +3906,7 @@
     </row>
     <row r="15" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="H15" s="18"/>
       <c r="J15" s="2" t="s">
@@ -3918,48 +3915,48 @@
     </row>
     <row r="16" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="B16" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="C16" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="D16" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="H16" s="16" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="B17" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="H17" s="16" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H18" s="16" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H19" s="16" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H20" s="16" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25"/>
@@ -3984,61 +3981,61 @@
     </row>
     <row r="29" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="B29" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="C29" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="D29" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="H29" s="16" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
     </row>
     <row r="30" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="B30" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="C30" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="D30" s="7" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="H30" s="16" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="31" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H31" s="16" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="32" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H32" s="16" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="33" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H33" s="16" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="34" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H34" s="16" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="35" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H35" s="16" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="36" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25"/>
@@ -4059,51 +4056,51 @@
     </row>
     <row r="42" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="B42" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="C42" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="D42" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="H42" s="16" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
     <row r="43" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="B43" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="C43" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D43" s="7" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="H43" s="16" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H44" s="16" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="45" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H45" s="16" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="46" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H46" s="16" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="47" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25"/>
@@ -4126,51 +4123,51 @@
     </row>
     <row r="55" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="B55" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="C55" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="D55" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="H55" s="16" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
     </row>
     <row r="56" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="B56" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C56" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="D56" s="7" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="H56" s="16" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="57" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H57" s="16" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="58" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H58" s="16" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="59" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H59" s="16" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="60" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25"/>
@@ -4184,7 +4181,7 @@
     </row>
     <row r="67" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="H67" s="18"/>
       <c r="J67" s="2" t="s">
@@ -4193,51 +4190,51 @@
     </row>
     <row r="68" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="B68" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="C68" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="D68" s="7" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="H68" s="16" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="69" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="B69" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C69" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="D69" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="H69" s="16" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="70" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H70" s="16" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="71" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H71" s="16" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="72" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H72" s="16" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="73" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25"/>
@@ -4251,7 +4248,7 @@
     </row>
     <row r="80" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="H80" s="18"/>
       <c r="J80" s="2" t="s">
@@ -4260,51 +4257,51 @@
     </row>
     <row r="81" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B81" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C81" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="D81" s="7" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="H81" s="16" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
     </row>
     <row r="82" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B82" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C82" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="D82" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="H82" s="16" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="83" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H83" s="16" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="84" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H84" s="16" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="85" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H85" s="16" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="86" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25"/>
@@ -4318,7 +4315,7 @@
     </row>
     <row r="93" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A93" s="2" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="H93" s="18"/>
       <c r="J93" s="2" t="s">
@@ -4327,54 +4324,54 @@
     </row>
     <row r="94" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="B94" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C94" s="7" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="D94" s="7" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="H94" s="16" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="I94" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
     </row>
     <row r="95" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="B95" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="C95" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="D95" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="H95" s="16" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="96" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H96" s="16" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="97" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H97" s="16" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="98" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H98" s="16" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="99" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25"/>
@@ -4388,7 +4385,7 @@
     </row>
     <row r="106" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A106" s="2" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="H106" s="18"/>
       <c r="J106" s="2" t="s">
@@ -4397,54 +4394,60 @@
     </row>
     <row r="107" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B107" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C107" t="s">
-        <v>419</v>
+        <v>258</v>
       </c>
       <c r="D107" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="H107" s="16" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="108" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B108" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C108" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="H108" s="16" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="109" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>307</v>
+      </c>
       <c r="C109" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="H109" s="16" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="110" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>307</v>
+      </c>
       <c r="C110" t="s">
         <v>250</v>
       </c>
       <c r="H110" s="16" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="111" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="H111" s="16" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="112" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25"/>
@@ -4477,57 +4480,60 @@
     </row>
     <row r="124" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C124" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="E124" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="G124" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="I124" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="125" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="E125" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="G125" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="126" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="E126" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="G126" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
     </row>
     <row r="127" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="E127" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="G127" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="128" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="A128" t="s">
+        <v>298</v>
+      </c>
+      <c r="G128" t="s">
         <v>491</v>
-      </c>
-    </row>
-    <row r="128" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="G128" t="s">
-        <v>492</v>
       </c>
     </row>
     <row r="129" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25"/>
@@ -4550,35 +4556,35 @@
     </row>
     <row r="137" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C137" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="E137" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="G137" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="138" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="E138" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="G138" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
     </row>
     <row r="139" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="E139" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="140" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25"/>
@@ -4603,38 +4609,38 @@
     </row>
     <row r="150" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C150" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="E150" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="G150" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
     </row>
     <row r="151" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="E151" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="G151" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
     </row>
     <row r="152" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="E152" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="G152" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
     </row>
     <row r="153" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25"/>
@@ -4659,29 +4665,29 @@
     </row>
     <row r="163" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="C163" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="E163" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="164" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="E164" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="165" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="E165" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="166" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25"/>
@@ -4697,7 +4703,7 @@
     </row>
     <row r="175" spans="1:10" s="13" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A175" s="13" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="H175" s="20"/>
       <c r="J175" s="13" t="s">
@@ -4706,32 +4712,32 @@
     </row>
     <row r="176" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="C176" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="E176" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="G176" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
     </row>
     <row r="177" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="E177" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="178" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="E178" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="179" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25"/>
@@ -4747,7 +4753,7 @@
     </row>
     <row r="188" spans="1:10" s="13" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A188" s="13" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="H188" s="20"/>
       <c r="J188" s="13" t="s">
@@ -4756,32 +4762,32 @@
     </row>
     <row r="189" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="C189" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="E189" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="I189" s="15" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
     </row>
     <row r="190" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="E190" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="191" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="E191" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="192" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25"/>
@@ -4797,7 +4803,7 @@
     </row>
     <row r="201" spans="1:10" s="13" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A201" s="13" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="H201" s="20"/>
       <c r="J201" s="13" t="s">
@@ -4806,29 +4812,29 @@
     </row>
     <row r="202" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="C202" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="E202" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="203" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="E203" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="204" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="E204" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="205" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25"/>
@@ -4844,7 +4850,7 @@
     </row>
     <row r="214" spans="1:10" s="13" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A214" s="13" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="H214" s="20"/>
       <c r="J214" s="13" t="s">
@@ -4853,7 +4859,7 @@
     </row>
     <row r="215" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="216" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25"/>
@@ -4880,7 +4886,7 @@
     </row>
     <row r="230" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A230" s="10" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="H230" s="21"/>
       <c r="J230" s="10" t="s">
@@ -4892,7 +4898,7 @@
         <v>115</v>
       </c>
       <c r="C231" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="232" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -4900,7 +4906,7 @@
         <v>115</v>
       </c>
       <c r="C232" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="233" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -4908,7 +4914,7 @@
         <v>115</v>
       </c>
       <c r="C233" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="234" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25"/>
@@ -4933,16 +4939,16 @@
     </row>
     <row r="244" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="C244" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="E244" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="I244" s="15" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
     </row>
     <row r="245" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25"/>
@@ -4960,7 +4966,7 @@
     </row>
     <row r="256" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A256" s="10" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="H256" s="21"/>
       <c r="J256" s="10" t="s">
@@ -4969,16 +4975,16 @@
     </row>
     <row r="257" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="C257" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="E257" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="I257" s="15" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="258" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25"/>
@@ -5008,7 +5014,7 @@
         <v>146</v>
       </c>
       <c r="C270" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="271" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -5016,7 +5022,7 @@
         <v>146</v>
       </c>
       <c r="C271" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="272" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
@@ -5024,7 +5030,7 @@
         <v>146</v>
       </c>
       <c r="C272" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="273" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25"/>
@@ -5086,7 +5092,7 @@
     </row>
     <row r="308" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A308" s="10" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="H308" s="21"/>
       <c r="J308" s="10" t="s">
@@ -5118,10 +5124,10 @@
     </row>
     <row r="322" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A322" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="C322" t="s">
-        <v>255</v>
+        <v>451</v>
       </c>
     </row>
     <row r="323" spans="1:10" ht="14.45" outlineLevel="1" x14ac:dyDescent="0.25"/>
@@ -5246,7 +5252,7 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="B1" t="s">
         <v>243</v>
@@ -7285,7 +7291,7 @@
         <v>#LastUsedPurpose_Balance_BeforeFirstUse</v>
       </c>
       <c r="C89" t="str">
-        <v>#StartMassRDY</v>
+        <v>#StartMass_RDY</v>
       </c>
       <c r="D89" t="str">
         <v>#LastUsedTime_Balance</v>
@@ -7324,8 +7330,8 @@
       </c>
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A91">
-        <v>0</v>
+      <c r="A91" t="str">
+        <v>#Balance</v>
       </c>
       <c r="B91">
         <v>0</v>
@@ -7347,8 +7353,8 @@
       </c>
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A92">
-        <v>0</v>
+      <c r="A92" t="str">
+        <v>#Balance</v>
       </c>
       <c r="B92">
         <v>0</v>
@@ -7647,8 +7653,8 @@
       </c>
     </row>
     <row r="105" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A105">
-        <v>0</v>
+      <c r="A105" t="str">
+        <v>#LiquidPhase</v>
       </c>
       <c r="B105">
         <v>0</v>
@@ -11372,7 +11378,7 @@
         <v>0</v>
       </c>
       <c r="C266" t="str">
-        <v>#FinalMassRDEt</v>
+        <v>#FinalMass_RDEt</v>
       </c>
       <c r="D266">
         <v>0</v>
@@ -12399,47 +12405,47 @@
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="B1" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="C1" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="D1" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="E1" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="B2" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="K2" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="B4" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="C4" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="L4" s="14" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="M4" s="14"/>
       <c r="N4" s="14"/>
@@ -12447,16 +12453,16 @@
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="K5" s="5"/>
       <c r="L5" s="5" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="M5" s="5" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="N5" s="5" t="s">
         <v>90</v>
       </c>
       <c r="O5" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="Q5" t="s">
         <v>243</v>
@@ -12464,22 +12470,22 @@
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="B6" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="E6" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="K6" s="11" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="L6" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="M6" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="Q6" t="s">
         <v>241</v>
@@ -12487,22 +12493,22 @@
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>458</v>
+      </c>
+      <c r="B7" t="s">
+        <v>463</v>
+      </c>
+      <c r="E7" t="s">
+        <v>462</v>
+      </c>
+      <c r="K7" s="11" t="s">
+        <v>461</v>
+      </c>
+      <c r="L7" t="s">
+        <v>460</v>
+      </c>
+      <c r="M7" t="s">
         <v>459</v>
-      </c>
-      <c r="B7" t="s">
-        <v>464</v>
-      </c>
-      <c r="E7" t="s">
-        <v>463</v>
-      </c>
-      <c r="K7" s="11" t="s">
-        <v>462</v>
-      </c>
-      <c r="L7" t="s">
-        <v>461</v>
-      </c>
-      <c r="M7" t="s">
-        <v>460</v>
       </c>
       <c r="Q7" t="s">
         <v>239</v>
@@ -12510,25 +12516,25 @@
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="B8" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="E8" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="K8" s="11" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="L8" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="M8" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="N8" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="Q8" t="s">
         <v>237</v>
@@ -12539,13 +12545,13 @@
         <v>250</v>
       </c>
       <c r="B9" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="K9" s="11" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="M9" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="Q9" t="s">
         <v>235</v>
@@ -12553,16 +12559,16 @@
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="B10" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="K10" s="11" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="M10" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="Q10" t="s">
         <v>233</v>
@@ -12570,13 +12576,13 @@
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B11" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="K11" s="11" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="M11" t="s">
         <v>241</v>
@@ -12584,10 +12590,10 @@
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B12" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="K12" s="11" t="s">
         <v>89</v>
@@ -12595,10 +12601,10 @@
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B13" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="K13" s="11" t="s">
         <v>248</v>
@@ -12606,141 +12612,141 @@
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B14" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="K14" s="11" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="L14" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="M14" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="N14" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="O14" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="B15" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="E15" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="K15" s="11" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="N15" t="s">
         <v>243</v>
       </c>
       <c r="O15" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="B16" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="K16" s="11" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B17" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="D17" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="K17" s="11" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="M17" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="B18" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="E18" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="K18" s="11" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="M18" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="N18" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="B19" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="K19" s="11" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="N19" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="O19" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="B20" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="K20" s="11" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="M20" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="N20" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="B21" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="D21" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="K21" s="11" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="M21" t="s">
         <v>233</v>
@@ -12748,19 +12754,19 @@
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="B22" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="K22" s="11" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="L22" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="M22" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="N22" t="s">
         <v>239</v>
@@ -12768,223 +12774,223 @@
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="E23" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="B24" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="E24" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="B25" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="E25" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="B26" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="E26" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="B27" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="E27" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="B28" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="E28" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="B29" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="B30" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="B31" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.25">
       <c r="E32" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="B33" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="E33" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="B34" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="E34" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="B35" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="B36" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="B37" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="E37" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="B38" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B39" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="B40" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="B41" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="B42" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="B43" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B44" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="B45" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="B46" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="B47" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Template Excel für Classes and Properties erstellt
</commit_message>
<xml_diff>
--- a/CASESTUDY_Hydrogenation.xlsx
+++ b/CASESTUDY_Hydrogenation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://universityofcambridgecloud-my.sharepoint.com/personal/lf576_cam_ac_uk/Documents/04_Coding/hydrogenation/current_versions/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="82" documentId="8_{3CA0C22B-1C3C-468B-A8A4-EC46740A7B5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BF7C0A2E-C8D9-446A-BC72-41ADC02F7BB1}"/>
+  <xr:revisionPtr revIDLastSave="86" documentId="8_{3CA0C22B-1C3C-468B-A8A4-EC46740A7B5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F3A68B46-3FC5-4FA3-93A6-BEB0CEDDED5D}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="3" xr2:uid="{D5389695-9B6E-4686-BC98-C44AC3042CAD}"/>
   </bookViews>
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="864" uniqueCount="492">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="866" uniqueCount="494">
   <si>
     <t>This is the file containing all the information about the Hydrogenation Process Case Study</t>
   </si>
@@ -1542,6 +1542,12 @@
   </si>
   <si>
     <t>#Reaction3</t>
+  </si>
+  <si>
+    <t>Wurde nicht eingetragen</t>
+  </si>
+  <si>
+    <t>Vll weil die Beziehung auch in die andere Richtung geht?</t>
   </si>
 </sst>
 </file>
@@ -1583,7 +1589,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1638,6 +1644,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -1660,7 +1672,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -1690,6 +1702,7 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -4183,6 +4196,9 @@
       <c r="A67" s="2" t="s">
         <v>331</v>
       </c>
+      <c r="C67" s="2" t="s">
+        <v>493</v>
+      </c>
       <c r="H67" s="18"/>
       <c r="J67" s="2" t="s">
         <v>90</v>
@@ -4195,7 +4211,7 @@
       <c r="B68" t="s">
         <v>329</v>
       </c>
-      <c r="C68" t="s">
+      <c r="C68" s="23" t="s">
         <v>314</v>
       </c>
       <c r="D68" s="7" t="s">
@@ -4212,7 +4228,7 @@
       <c r="B69" t="s">
         <v>327</v>
       </c>
-      <c r="C69" t="s">
+      <c r="C69" s="23" t="s">
         <v>326</v>
       </c>
       <c r="D69" t="s">
@@ -4250,6 +4266,9 @@
       <c r="A80" s="2" t="s">
         <v>324</v>
       </c>
+      <c r="C80" s="2" t="s">
+        <v>492</v>
+      </c>
       <c r="H80" s="18"/>
       <c r="J80" s="2" t="s">
         <v>90</v>
@@ -4262,7 +4281,7 @@
       <c r="B81" t="s">
         <v>322</v>
       </c>
-      <c r="C81" t="s">
+      <c r="C81" s="23" t="s">
         <v>314</v>
       </c>
       <c r="D81" s="7" t="s">
@@ -4279,7 +4298,7 @@
       <c r="B82" t="s">
         <v>320</v>
       </c>
-      <c r="C82" t="s">
+      <c r="C82" s="23" t="s">
         <v>319</v>
       </c>
       <c r="D82" t="s">

</xml_diff>